<commit_message>
rocphotos: constrain oa:motivatedBy to an ItemList holding oa:identifying
The motivation list existed but nothing used it. oa:motivatedBy now takes
its range from #itemlist_motivation, and the profile describes the
oa:identifying entity (same as in the oa: schema), which a crate must
carry, as with any ItemList value. Using a list leaves room for more
motivations later. Profile text updated; the motivatedBy known gap is gone.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/profiles/rocphotos/profile-crate/ro-crate-metadata.xlsx
+++ b/profiles/rocphotos/profile-crate/ro-crate-metadata.xlsx
@@ -13,13 +13,14 @@
     <sheet sheetId="7" name="@type=rdfs_Class" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="@type=rdf_Property" state="visible" r:id="rId11"/>
     <sheet sheetId="9" name="@type=ItemList" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="@type=oa_Motivation" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="296">
   <si>
     <t>Name</t>
   </si>
@@ -759,7 +760,10 @@
     <t>"http://www.w3.org/ns/oa#motivatedBy"</t>
   </si>
   <si>
-    <t>Always oa:identifying — the annotation says who this is. Left range-unconstrained: the validator resolves a range reference within the target crate, and rocphotos does not (yet) describe oa:identifying as an entity of its own.</t>
+    <t>Always oa:identifying — the annotation says who this is. The value comes from an ItemList so more motivations can be added later. As with any ItemList value, the crate must carry the oa:identifying entity itself, matching the one in this profile.</t>
+  </si>
+  <si>
+    <t>"#itemlist_motivation"</t>
   </si>
   <si>
     <t>#prop_standoff_writtenToFile</t>
@@ -892,6 +896,18 @@
   </si>
   <si>
     <t>"http://www.w3.org/ns/oa#identifying"</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#identifying</t>
+  </si>
+  <si>
+    <t>oa:Motivation</t>
+  </si>
+  <si>
+    <t>identifying</t>
+  </si>
+  <si>
+    <t>The motivation for when the user intends to assign an identity to the Target or identify what is being depicted or described in the Target.</t>
   </si>
 </sst>
 </file>
@@ -1377,6 +1393,48 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B4"/>
@@ -3012,34 +3070,37 @@
       <c r="G40" t="s">
         <v>246</v>
       </c>
+      <c r="H40" t="s">
+        <v>247</v>
+      </c>
       <c r="I40">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B41" t="s">
         <v>111</v>
       </c>
       <c r="C41" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D41" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E41" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F41" t="s">
         <v>231</v>
       </c>
       <c r="G41" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I41">
         <v>1</v>
@@ -3047,7 +3108,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B42" t="s">
         <v>111</v>
@@ -3065,7 +3126,7 @@
         <v>242</v>
       </c>
       <c r="G42" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H42" t="s">
         <v>195</v>
@@ -3076,7 +3137,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B43" t="s">
         <v>111</v>
@@ -3094,7 +3155,7 @@
         <v>158</v>
       </c>
       <c r="G43" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H43" t="s">
         <v>115</v>
@@ -3105,25 +3166,25 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B44" t="s">
         <v>111</v>
       </c>
       <c r="C44" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D44" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E44" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F44" t="s">
         <v>158</v>
       </c>
       <c r="G44" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="H44" t="s">
         <v>115</v>
@@ -3134,7 +3195,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B45" t="s">
         <v>111</v>
@@ -3149,10 +3210,10 @@
         <v>112</v>
       </c>
       <c r="F45" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G45" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H45" t="s">
         <v>115</v>
@@ -3163,7 +3224,7 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B46" t="s">
         <v>111</v>
@@ -3178,10 +3239,10 @@
         <v>161</v>
       </c>
       <c r="F46" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G46" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H46" t="s">
         <v>192</v>
@@ -3189,25 +3250,25 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B47" t="s">
         <v>111</v>
       </c>
       <c r="C47" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D47" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E47" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F47" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G47" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H47" t="s">
         <v>115</v>
@@ -3218,25 +3279,25 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B48" t="s">
         <v>111</v>
       </c>
       <c r="C48" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D48" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E48" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F48" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G48" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H48" t="s">
         <v>115</v>
@@ -3244,25 +3305,25 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B49" t="s">
         <v>111</v>
       </c>
       <c r="C49" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D49" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E49" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F49" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G49" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H49" t="s">
         <v>153</v>
@@ -3273,25 +3334,25 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B50" t="s">
         <v>111</v>
       </c>
       <c r="C50" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D50" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E50" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F50" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G50" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H50" t="s">
         <v>115</v>
@@ -3302,25 +3363,25 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B51" t="s">
         <v>111</v>
       </c>
       <c r="C51" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D51" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E51" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F51" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G51" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="H51" t="s">
         <v>115</v>
@@ -3357,24 +3418,24 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>